<commit_message>
Updated the calibration data to match the 4 legs
</commit_message>
<xml_diff>
--- a/Servo_test/Servo Calibration.xlsx
+++ b/Servo_test/Servo Calibration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Paarth\Project_Arachnid\Servo_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3753738-60F7-4AB3-B13E-58F7312BEB1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D30942-C777-4C4E-9F38-2F23B75CF0E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{C59693A6-8C39-4E44-9FD9-EFF308F04AC1}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="16090" xr2:uid="{C59693A6-8C39-4E44-9FD9-EFF308F04AC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
   <si>
     <t xml:space="preserve">SERVO MODEL </t>
   </si>
@@ -71,12 +71,6 @@
     <t>Front - Right</t>
   </si>
   <si>
-    <t>Middle - Left</t>
-  </si>
-  <si>
-    <t>Middle - Right</t>
-  </si>
-  <si>
     <t>Rear - Left</t>
   </si>
   <si>
@@ -92,12 +86,6 @@
     <t>Tibia</t>
   </si>
   <si>
-    <t xml:space="preserve">Coxa </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Femur </t>
-  </si>
-  <si>
     <t>MG958</t>
   </si>
   <si>
@@ -129,9 +117,6 @@
   </si>
   <si>
     <t>~180</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#Note: estimate an offset of  -1&lt;=x&lt;=2 degrees </t>
   </si>
   <si>
     <t>~150-160</t>
@@ -141,17 +126,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -170,7 +148,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,18 +182,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -273,19 +239,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -304,26 +270,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -658,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF4F2058-E9F9-4B44-BAAE-88291276ADE5}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
@@ -690,7 +642,7 @@
         <v>3</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>1</v>
@@ -711,11 +663,11 @@
       <c r="B3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>14</v>
+      <c r="C3" s="14" t="s">
+        <v>12</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E3" s="9">
         <v>500</v>
@@ -724,84 +676,83 @@
         <v>2500</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="M3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="8">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="9">
+        <v>620</v>
+      </c>
+      <c r="F4" s="9">
+        <v>2380</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="10">
-        <v>2</v>
-      </c>
-      <c r="B4" s="11" t="s">
+      <c r="N4" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="8">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C5" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="11">
+      <c r="E5" s="9">
         <v>620</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F5" s="9">
         <v>2380</v>
       </c>
-      <c r="L4" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" s="10">
-        <v>3</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="11">
-        <v>620</v>
-      </c>
-      <c r="F5" s="11">
-        <v>2380</v>
-      </c>
       <c r="L5" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
-      <c r="C6" s="27"/>
       <c r="L6" s="6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -811,11 +762,11 @@
       <c r="B7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="26" t="s">
-        <v>14</v>
+      <c r="C7" s="19" t="s">
+        <v>12</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E7" s="9">
         <v>500</v>
@@ -824,13 +775,13 @@
         <v>2500</v>
       </c>
       <c r="L7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="M7" s="6" t="s">
-        <v>27</v>
-      </c>
       <c r="N7" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -840,11 +791,11 @@
       <c r="B8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>15</v>
+      <c r="C8" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E8" s="11">
         <v>620</v>
@@ -860,11 +811,11 @@
       <c r="B9" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>20</v>
       </c>
       <c r="E9" s="11">
         <v>620</v>
@@ -875,7 +826,6 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
-      <c r="C10" s="27"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
@@ -884,11 +834,11 @@
       <c r="B11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="26" t="s">
-        <v>17</v>
+      <c r="C11" s="19" t="s">
+        <v>12</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E11" s="9">
         <v>500</v>
@@ -896,58 +846,49 @@
       <c r="F11" s="9">
         <v>2500</v>
       </c>
-      <c r="L11" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="M11" s="29"/>
-      <c r="N11" s="29"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A12" s="10">
+      <c r="A12" s="12">
         <v>8</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="11">
-        <v>620</v>
-      </c>
-      <c r="F12" s="11">
-        <v>2380</v>
-      </c>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
+      <c r="C12" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="13">
+        <v>600</v>
+      </c>
+      <c r="F12" s="13">
+        <v>2400</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="10">
+      <c r="A13" s="12">
         <v>9</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="11">
-        <v>620</v>
-      </c>
-      <c r="F13" s="11">
-        <v>2380</v>
+      <c r="C13" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="13">
+        <v>600</v>
+      </c>
+      <c r="F13" s="13">
+        <v>2400</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
-      <c r="C14" s="27"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
@@ -956,11 +897,11 @@
       <c r="B15" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>14</v>
+      <c r="C15" s="19" t="s">
+        <v>12</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E15" s="9">
         <v>500</v>
@@ -970,175 +911,47 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A16" s="8">
+      <c r="A16" s="10">
         <v>11</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="9">
+      <c r="C16" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="11">
         <v>500</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="11">
         <v>2500</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="8">
+      <c r="A17" s="10">
         <v>12</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="9">
-        <v>500</v>
-      </c>
-      <c r="F17" s="9">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="4"/>
-      <c r="C18" s="27"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="8">
-        <v>13</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="9">
-        <v>500</v>
-      </c>
-      <c r="F19" s="9">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="12">
-        <v>14</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E20" s="13">
-        <v>600</v>
-      </c>
-      <c r="F20" s="13">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="12">
-        <v>15</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" s="13">
-        <v>600</v>
-      </c>
-      <c r="F21" s="13">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="4"/>
-      <c r="C22" s="27"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="8">
-        <v>16</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="9">
-        <v>500</v>
-      </c>
-      <c r="F23" s="9">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="14">
-        <v>17</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="15">
-        <v>500</v>
-      </c>
-      <c r="F24" s="15">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="16">
-        <v>18</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="E25" s="17">
+      <c r="E17" s="11">
         <v>750</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F17" s="11">
         <v>2250</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>